<commit_message>
docs: conclui entrega da ficha unica
Registra a validação local e no QAS, documenta o modo de serviço e corrige as instruções da ficha.

Co-authored-by: Copilot <223556219+Copilot@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/src/anuncio_navio/recursos/ficha_modelo.xlsx
+++ b/src/anuncio_navio/recursos/ficha_modelo.xlsx
@@ -1142,14 +1142,14 @@
     <row r="9">
       <c r="A9" s="18" t="inlineStr">
         <is>
-          <t>Pronto: devolva ESTE arquivo. O número da viagem e a classificação da operação são definidos no processamento.</t>
+          <t>Ao terminar: salve (Cmd+S) e feche esta planilha. O robô processa o arquivo automaticamente; não é necessário devolvê-lo.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="18" t="inlineStr">
         <is>
-          <t>Ao terminar: salve (Cmd+S) e feche. O robô devolve o resultado na linha STATUS e prepara a próxima ficha.</t>
+          <t>Em caso de erro, o motivo aparece na linha STATUS. Corrija os campos indicados e salve novamente.</t>
         </is>
       </c>
     </row>

</xml_diff>